<commit_message>
chore: removed jorge and ivan, added anamaria
</commit_message>
<xml_diff>
--- a/public/data/info.xlsx
+++ b/public/data/info.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\cisdeli\Purdue\CiampittiLab\ciampitti-lab.github.io\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94A2929E-2AE6-4260-88EA-9E9A57F4DF9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65A8A05A-A465-412B-BC4B-82AA31ABD11A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{680A29BD-E113-4DFE-A325-D924D35BBF8F}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="171">
   <si>
     <t>role</t>
   </si>
@@ -449,18 +449,6 @@
     <t>Short series documenting Pedro Cisdeli's hands-on journey building ag-tech tools for Apple Vision Pro</t>
   </si>
   <si>
-    <t>jorge_jola.jpg</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/in/jjola-unal/</t>
-  </si>
-  <si>
-    <t>Jorge Jola</t>
-  </si>
-  <si>
-    <t>Undergraduate student in Agronomic Engineering at the National University of Colombia, with experience in agronomic data analysis. Skilled in statistics, Web applications, and the application of machine learning in agriculture.</t>
-  </si>
-  <si>
     <t>Norman Menocal</t>
   </si>
   <si>
@@ -470,15 +458,6 @@
     <t>I am an agronomist interested in sustainable agriculture and the use of new technologies to improve the yield of agronomic crops. I have hands-on experience in fields crops, data collection, harvesting and pesticides applications, gained through academic projects and internship.</t>
   </si>
   <si>
-    <t>ivan_mejia.jpg</t>
-  </si>
-  <si>
-    <t>Data Science student at Universidad del Norte (Barranquilla, Colombia). Focused on leveraging data analysis and processing tools using Python for knowledge extraction. Passionate about using data-driven solutions to solve real-world problems and improve people's quality of life through the advancement of digital agriculture.</t>
-  </si>
-  <si>
-    <t>Ivan Ramirez</t>
-  </si>
-  <si>
     <t>Agronomist researching cropping systems and farmer decision-making, integrating remote sensing and digital agriculture to evaluate how technological innovation and environmental variability influence agricultural sustainability and productivity.</t>
   </si>
   <si>
@@ -561,6 +540,18 @@
   </si>
   <si>
     <t>Senior Data Scientist</t>
+  </si>
+  <si>
+    <t>Anamaria Rodriguez Ramirez</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/anamaria-rodriguez-ramirez/</t>
+  </si>
+  <si>
+    <t>Undergraduate student of Agronomic Engineering at the Universidad Nacional de Colombia, with experience in research and data analysis in phytopathology and physiology. </t>
+  </si>
+  <si>
+    <t>anamaria.jpg</t>
   </si>
 </sst>
 </file>
@@ -946,7 +937,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87EB64B1-8415-484E-B4A1-A632CC3BB222}">
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
@@ -1034,7 +1025,7 @@
         <v>37</v>
       </c>
       <c r="F4" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1085,7 +1076,7 @@
         <v>11</v>
       </c>
       <c r="C7" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="D7" t="s">
         <v>101</v>
@@ -1131,7 +1122,7 @@
         <v>40</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1139,19 +1130,19 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="C10" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="D10" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="F10" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -1159,19 +1150,19 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>148</v>
+        <v>167</v>
       </c>
       <c r="C11" t="s">
         <v>2</v>
       </c>
       <c r="D11" t="s">
-        <v>149</v>
-      </c>
-      <c r="E11" t="s">
-        <v>150</v>
+        <v>170</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>168</v>
       </c>
       <c r="F11" t="s">
-        <v>151</v>
+        <v>169</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -1179,16 +1170,19 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>13</v>
+        <v>141</v>
       </c>
       <c r="C12" t="s">
         <v>2</v>
       </c>
       <c r="D12" t="s">
-        <v>103</v>
+        <v>142</v>
+      </c>
+      <c r="E12" t="s">
+        <v>143</v>
       </c>
       <c r="F12" t="s">
-        <v>31</v>
+        <v>144</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -1196,16 +1190,19 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>145</v>
+        <v>13</v>
       </c>
       <c r="C13" t="s">
         <v>2</v>
       </c>
       <c r="D13" t="s">
-        <v>143</v>
+        <v>103</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>168</v>
       </c>
       <c r="F13" t="s">
-        <v>144</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -1213,39 +1210,39 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>138</v>
+        <v>152</v>
       </c>
       <c r="C14" t="s">
         <v>2</v>
       </c>
       <c r="D14" t="s">
-        <v>136</v>
+        <v>147</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>137</v>
+        <v>153</v>
       </c>
       <c r="F14" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="12" customHeight="1">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C15" t="s">
         <v>2</v>
       </c>
       <c r="D15" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="F15" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -1253,19 +1250,16 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>165</v>
+        <v>136</v>
       </c>
       <c r="C16" t="s">
         <v>2</v>
       </c>
       <c r="D16" t="s">
-        <v>156</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>163</v>
+        <v>137</v>
       </c>
       <c r="F16" t="s">
-        <v>164</v>
+        <v>138</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -1273,16 +1267,19 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="C17" t="s">
         <v>2</v>
       </c>
       <c r="D17" t="s">
-        <v>141</v>
+        <v>146</v>
+      </c>
+      <c r="E17" t="s">
+        <v>151</v>
       </c>
       <c r="F17" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -1290,19 +1287,19 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>152</v>
+        <v>115</v>
       </c>
       <c r="C18" t="s">
         <v>2</v>
       </c>
       <c r="D18" t="s">
-        <v>153</v>
-      </c>
-      <c r="E18" t="s">
-        <v>158</v>
+        <v>116</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>123</v>
       </c>
       <c r="F18" t="s">
-        <v>157</v>
+        <v>117</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -1310,19 +1307,19 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>115</v>
+        <v>12</v>
       </c>
       <c r="C19" t="s">
         <v>2</v>
       </c>
       <c r="D19" t="s">
-        <v>116</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>123</v>
+        <v>100</v>
+      </c>
+      <c r="E19" t="s">
+        <v>41</v>
       </c>
       <c r="F19" t="s">
-        <v>117</v>
+        <v>30</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -1330,39 +1327,19 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>12</v>
+        <v>159</v>
       </c>
       <c r="C20" t="s">
         <v>2</v>
       </c>
       <c r="D20" t="s">
-        <v>100</v>
-      </c>
-      <c r="E20" t="s">
-        <v>41</v>
+        <v>148</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>160</v>
       </c>
       <c r="F20" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6">
-      <c r="A21">
-        <v>20</v>
-      </c>
-      <c r="B21" t="s">
-        <v>166</v>
-      </c>
-      <c r="C21" t="s">
-        <v>2</v>
-      </c>
-      <c r="D21" t="s">
         <v>155</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="F21" t="s">
-        <v>162</v>
       </c>
     </row>
   </sheetData>
@@ -1371,12 +1348,13 @@
     <hyperlink ref="E2" r:id="rId2" xr:uid="{A94255E5-8ECE-483E-BE8F-EE9B37DAE260}"/>
     <hyperlink ref="E4" r:id="rId3" xr:uid="{F9808E56-71B8-4EF9-927B-9D68DAE7673D}"/>
     <hyperlink ref="E7" r:id="rId4" xr:uid="{2A6658AF-7FC0-4FB5-9A94-14DD4D416741}"/>
-    <hyperlink ref="E19" r:id="rId5" xr:uid="{D4CFB1C7-1AE1-491B-850A-B6BFAE8BB6A7}"/>
-    <hyperlink ref="E14" r:id="rId6" tooltip="https://www.linkedin.com/in/jjola-unal/" xr:uid="{9B18B642-568C-42D5-8EB7-C9BF52A122A6}"/>
-    <hyperlink ref="E15" r:id="rId7" xr:uid="{AEE5542A-4545-4E11-B4D0-8CB3A09EDB67}"/>
-    <hyperlink ref="E16" r:id="rId8" xr:uid="{275E1803-2201-4510-93DA-AF5897C61F6B}"/>
-    <hyperlink ref="E21" r:id="rId9" xr:uid="{6CD67109-5E4B-4530-B2D9-396F2CAFB8B1}"/>
-    <hyperlink ref="E10" r:id="rId10" xr:uid="{E9C7984C-B4B0-4DF0-82E3-259B124343A1}"/>
+    <hyperlink ref="E20" r:id="rId5" xr:uid="{6CD67109-5E4B-4530-B2D9-396F2CAFB8B1}"/>
+    <hyperlink ref="E10" r:id="rId6" xr:uid="{E9C7984C-B4B0-4DF0-82E3-259B124343A1}"/>
+    <hyperlink ref="E15" r:id="rId7" xr:uid="{275E1803-2201-4510-93DA-AF5897C61F6B}"/>
+    <hyperlink ref="E14" r:id="rId8" xr:uid="{AEE5542A-4545-4E11-B4D0-8CB3A09EDB67}"/>
+    <hyperlink ref="E18" r:id="rId9" xr:uid="{D4CFB1C7-1AE1-491B-850A-B6BFAE8BB6A7}"/>
+    <hyperlink ref="E11" r:id="rId10" tooltip="https://www.linkedin.com/in/anamaria-rodriguez-ramirez/" xr:uid="{FEB70905-ECEF-48C9-AB8A-6FB9A18013E7}"/>
+    <hyperlink ref="E13" r:id="rId11" tooltip="https://www.linkedin.com/in/anamaria-rodriguez-ramirez/" xr:uid="{FA066E13-EED7-4A4D-8BC8-71E95FF896AB}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>